<commit_message>
Autoelektrika: přidán startér (kalkulačka, tabulka průřezů) do webu, Excelu i PDF
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018zchM4LA7BGGwBFTWSip3W
</commit_message>
<xml_diff>
--- a/autoelektrika/Pomucka_autoelektrika.xlsx
+++ b/autoelektrika/Pomucka_autoelektrika.xlsx
@@ -11,14 +11,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Úbytek a průřez" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pojistka a kabel" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Výkon a proud" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baterie" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zdroje a měniče" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energetická bilance" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabulky" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check nový okruh" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check diagnostika" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check ostrovní systém" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startér" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baterie" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zdroje a měniče" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energetická bilance" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabulky" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check nový okruh" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check diagnostika" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check ostrovní systém" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,10 +28,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -124,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -163,17 +165,20 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="3" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -598,7 +603,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Kabely a jištění: Úbytek a průřez | Pojistka a kabel | Výkon a proud (srovnání 12/24/48 V)</t>
+          <t>Kabely a jištění: Úbytek a průřez | Pojistka a kabel | Výkon a proud (srovnání 12/24/48 V) | Startér</t>
         </is>
       </c>
     </row>
@@ -660,6 +665,162 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Check nový okruh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Instalace nového spotřebiče / okruhu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Bod</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>Splněno (x)</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>Poznámka</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Určen trvalý a špičkový proud spotřebiče</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="n"/>
+      <c r="C5" s="8" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Pojistka nebo jistič co nejblíž ke zdroji (baterii), dimenzovaná na kabel</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="n"/>
+      <c r="C6" s="8" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Průřez zkontrolován na úbytek napětí i na trvalý proud</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="n"/>
+      <c r="C7" s="8" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>Kabel odolný teplu a oděru, ochranný vlnovec, průchodky v plechu</t>
+        </is>
+      </c>
+      <c r="B8" s="28" t="n"/>
+      <c r="C8" s="8" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>Kvalitní lisované koncovky a spoje, správná velikost oka</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="n"/>
+      <c r="C9" s="8" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>Velké zátěže spínány přes relé / stykač</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="n"/>
+      <c r="C10" s="8" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Kostrový spoj čistý, kov na kov, zajištěn proti uvolnění</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="n"/>
+      <c r="C11" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>Spoje utaženy předepsaným momentem, svorky zakryty proti zkratu</t>
+        </is>
+      </c>
+      <c r="B12" s="28" t="n"/>
+      <c r="C12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>Změřen úbytek napětí na plus i mínus pod zátěží</t>
+        </is>
+      </c>
+      <c r="B13" s="28" t="n"/>
+      <c r="C13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>Zákres do schématu, kabely označeny</t>
+        </is>
+      </c>
+      <c r="B14" s="28" t="n"/>
+      <c r="C14" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="20">
+        <f>"Splněno "&amp;COUNTIF(B5:B14,"x")&amp;" z 10"</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A5:B14">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$B5="x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="B5 B6 B7 B8 B9 B10 B11 B12 B13 B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"x,"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -688,105 +849,105 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Bod</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Splněno (x)</t>
         </is>
       </c>
-      <c r="C4" s="24" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>Poznámka</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Vizuálně: svorky, koroze, uchycení, oleje, zápach</t>
         </is>
       </c>
-      <c r="B5" s="27" t="n"/>
+      <c r="B5" s="28" t="n"/>
       <c r="C5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>Napětí v klidu (po ≥ 4 h): ≥ 12,4 V (24 V: 24,8 V)</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n"/>
+      <c r="B6" s="28" t="n"/>
       <c r="C6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>Při startu napětí nesmí klesnout pod ≈ 9,6 V (24 V: 19,2 V)</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n"/>
+      <c r="B7" s="28" t="n"/>
       <c r="C7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>Napětí při běžícím motoru: 13,8–14,8 V (24 V: 27,6–29,6 V)</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n"/>
+      <c r="B8" s="28" t="n"/>
       <c r="C8" s="8" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="26" t="inlineStr">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>Úbytek napětí na kladném kabelu při startu: &lt; 0,5 V</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n"/>
+      <c r="B9" s="28" t="n"/>
       <c r="C9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="26" t="inlineStr">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t>Úbytek napětí na kostře při startu: &lt; 0,3 V</t>
         </is>
       </c>
-      <c r="B10" s="27" t="n"/>
+      <c r="B10" s="28" t="n"/>
       <c r="C10" s="8" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="26" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>Klidový odběr po uspání vozidla: typicky &lt; 50 mA (dle výrobce)</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n"/>
+      <c r="B11" s="28" t="n"/>
       <c r="C11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="26" t="inlineStr">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>Zvlnění alternátoru (AC) při chodu: &lt; 0,5 V</t>
         </is>
       </c>
-      <c r="B12" s="27" t="n"/>
+      <c r="B12" s="28" t="n"/>
       <c r="C12" s="8" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="26" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>Alternátor, řemen a pojistky nabíjecího okruhu OK</t>
         </is>
       </c>
-      <c r="B13" s="27" t="n"/>
+      <c r="B13" s="28" t="n"/>
       <c r="C13" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="24">
+      <c r="A15" s="20">
         <f>"Splněno "&amp;COUNTIF(B5:B13,"x")&amp;" z 9"</f>
         <v/>
       </c>
@@ -806,7 +967,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -835,123 +996,123 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Bod</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Splněno (x)</t>
         </is>
       </c>
-      <c r="C4" s="24" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>Poznámka</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Baterie s vhodným BMS / ochranami, ventilace u olova</t>
         </is>
       </c>
-      <c r="B5" s="27" t="n"/>
+      <c r="B5" s="28" t="n"/>
       <c r="C5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>Hlavní pojistka (MEGA / Class T) a hlavní vypínač u baterie</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n"/>
+      <c r="B6" s="28" t="n"/>
       <c r="C6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>Pro 48 V: pojistky, vypínače a relé s jmenovitým DC napětím ≥ 58 V</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n"/>
+      <c r="B7" s="28" t="n"/>
       <c r="C7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>Samostatná pojistka na každou větev paralelních baterií</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n"/>
+      <c r="B8" s="28" t="n"/>
       <c r="C8" s="8" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="26" t="inlineStr">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>Měření (shunt, BMS) zapojeno, nastavena kapacita a napětí</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n"/>
+      <c r="B9" s="28" t="n"/>
       <c r="C9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="26" t="inlineStr">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t>Solární regulátor nastaven na typ baterie, kontrola Voc za mrazu</t>
         </is>
       </c>
-      <c r="B10" s="27" t="n"/>
+      <c r="B10" s="28" t="n"/>
       <c r="C10" s="8" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="26" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>Střídač: DC kabel krátký a dostatečný, pojistka u baterie</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n"/>
+      <c r="B11" s="28" t="n"/>
       <c r="C11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="26" t="inlineStr">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>AC strana: RCD/jistič, ochrana a uzemnění dle typu aplikace</t>
         </is>
       </c>
-      <c r="B12" s="27" t="n"/>
+      <c r="B12" s="28" t="n"/>
       <c r="C12" s="8" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="26" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>Společná kostra / záporná sběrnice, jedno místo spojení s kostrou</t>
         </is>
       </c>
-      <c r="B13" s="27" t="n"/>
+      <c r="B13" s="28" t="n"/>
       <c r="C13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="26" t="inlineStr">
+      <c r="A14" s="27" t="inlineStr">
         <is>
           <t>Polarita a štítky na všech vodičích, zkušební zapnutí po částech</t>
         </is>
       </c>
-      <c r="B14" s="27" t="n"/>
+      <c r="B14" s="28" t="n"/>
       <c r="C14" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="26" t="inlineStr">
+      <c r="A15" s="27" t="inlineStr">
         <is>
           <t>Zátěžový test: výdrž, úbytky, teploty spojů</t>
         </is>
       </c>
-      <c r="B15" s="27" t="n"/>
+      <c r="B15" s="28" t="n"/>
       <c r="C15" s="8" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="24">
+      <c r="A17" s="20">
         <f>"Splněno "&amp;COUNTIF(B5:B15,"x")&amp;" z 11"</f>
         <v/>
       </c>
@@ -971,13 +1132,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -989,6 +1150,8 @@
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="3" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="3" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -999,7 +1162,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="29" t="inlineStr">
         <is>
           <t>mm²</t>
         </is>
@@ -1027,6 +1190,11 @@
       <c r="I2" s="5" t="inlineStr">
         <is>
           <t>E24</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Startér mm²</t>
         </is>
       </c>
     </row>
@@ -1049,6 +1217,9 @@
       <c r="I3" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="K3" s="8" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="n">
@@ -1069,6 +1240,9 @@
       <c r="I4" s="8" t="n">
         <v>1.1</v>
       </c>
+      <c r="K4" s="8" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="n">
@@ -1089,6 +1263,9 @@
       <c r="I5" s="8" t="n">
         <v>1.2</v>
       </c>
+      <c r="K5" s="8" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n">
@@ -1109,6 +1286,9 @@
       <c r="I6" s="8" t="n">
         <v>1.3</v>
       </c>
+      <c r="K6" s="8" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="n">
@@ -1129,6 +1309,9 @@
       <c r="I7" s="8" t="n">
         <v>1.5</v>
       </c>
+      <c r="K7" s="8" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n">
@@ -1143,6 +1326,9 @@
       <c r="I8" s="8" t="n">
         <v>1.6</v>
       </c>
+      <c r="K8" s="8" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n">
@@ -1157,6 +1343,9 @@
       <c r="I9" s="8" t="n">
         <v>1.8</v>
       </c>
+      <c r="K9" s="8" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
@@ -1171,6 +1360,9 @@
       <c r="I10" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="K10" s="8" t="n">
+        <v>120</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n">
@@ -1185,6 +1377,9 @@
       <c r="I11" s="8" t="n">
         <v>2.2</v>
       </c>
+      <c r="K11" s="8" t="n">
+        <v>150</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
@@ -1198,6 +1393,9 @@
       </c>
       <c r="I12" s="8" t="n">
         <v>2.4</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>185</v>
       </c>
     </row>
     <row r="13">
@@ -2538,6 +2736,487 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Startér</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Špičkový proud při startu; celkový úbytek na + i − kabelu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Vstupy</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>Min. průřez [mm²], 12 V, 0,5 V, 40 °C: řádky = A, sloupce = m (+ i −)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Napětí soustavy</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Startovací proud (špička)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F6" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E6*(1/56*(1+0.00393*(40-20)))*F$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="G6" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E6*(1/56*(1+0.00393*(40-20)))*G$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="H6" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E6*(1/56*(1+0.00393*(40-20)))*H$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="I6" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E6*(1/56*(1+0.00393*(40-20)))*I$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="J6" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E6*(1/56*(1+0.00393*(40-20)))*J$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="K6" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E6*(1/56*(1+0.00393*(40-20)))*K$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Délka kladného kabelu</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="F7" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E7*(1/56*(1+0.00393*(40-20)))*F$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="G7" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E7*(1/56*(1+0.00393*(40-20)))*G$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="H7" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E7*(1/56*(1+0.00393*(40-20)))*H$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="I7" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E7*(1/56*(1+0.00393*(40-20)))*I$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="J7" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E7*(1/56*(1+0.00393*(40-20)))*J$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="K7" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E7*(1/56*(1+0.00393*(40-20)))*K$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Délka záporného kabelu / kostry</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="F8" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E8*(1/56*(1+0.00393*(40-20)))*F$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="G8" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E8*(1/56*(1+0.00393*(40-20)))*G$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="H8" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E8*(1/56*(1+0.00393*(40-20)))*H$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="I8" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E8*(1/56*(1+0.00393*(40-20)))*I$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="J8" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E8*(1/56*(1+0.00393*(40-20)))*J$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="K8" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E8*(1/56*(1+0.00393*(40-20)))*K$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Povolený úbytek celkem (12 V: 0,5; 24 V: 1)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="F9" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E9*(1/56*(1+0.00393*(40-20)))*F$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="G9" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E9*(1/56*(1+0.00393*(40-20)))*G$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="H9" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E9*(1/56*(1+0.00393*(40-20)))*H$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="I9" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E9*(1/56*(1+0.00393*(40-20)))*I$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="J9" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E9*(1/56*(1+0.00393*(40-20)))*J$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="K9" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E9*(1/56*(1+0.00393*(40-20)))*K$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Teplota kabelu</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>400</v>
+      </c>
+      <c r="F10" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E10*(1/56*(1+0.00393*(40-20)))*F$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="G10" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E10*(1/56*(1+0.00393*(40-20)))*G$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="H10" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E10*(1/56*(1+0.00393*(40-20)))*H$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="I10" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E10*(1/56*(1+0.00393*(40-20)))*I$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="J10" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E10*(1/56*(1+0.00393*(40-20)))*J$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="K10" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E10*(1/56*(1+0.00393*(40-20)))*K$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Typicky: benzín 150–250 A, diesel 250–450 A, nákladní 24 V 400–800 A. Rozhoduje údaj výrobce motoru.</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>600</v>
+      </c>
+      <c r="F11" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E11*(1/56*(1+0.00393*(40-20)))*F$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="G11" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E11*(1/56*(1+0.00393*(40-20)))*G$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="H11" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E11*(1/56*(1+0.00393*(40-20)))*H$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="I11" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E11*(1/56*(1+0.00393*(40-20)))*I$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="J11" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E11*(1/56*(1+0.00393*(40-20)))*J$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+      <c r="K11" s="8">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$E11*(1/56*(1+0.00393*(40-20)))*K$5/0.5,0),0)),"&gt;185")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Výsledky</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Odpor smyčky (délka · ρ)</t>
+        </is>
+      </c>
+      <c r="B14" s="21">
+        <f>(1/56*(1+0.00393*($B$10-20)))*($B$7+$B$8)</f>
+        <v/>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Ω·mm²</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Vypočtený min. průřez</t>
+        </is>
+      </c>
+      <c r="B15" s="10">
+        <f>$B$6*$B$14/$B$9</f>
+        <v/>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>mm²</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Doporučený průřez (+ i −)</t>
+        </is>
+      </c>
+      <c r="B16" s="22">
+        <f>IFERROR(INDEX(Data!$K$3:$K$12,MATCH(TRUE,INDEX(Data!$K$3:$K$12&gt;=$B$15,0),0)),"&gt; 185 – paralelní kabely")</f>
+        <v/>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>mm²</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Úbytek při startu</t>
+        </is>
+      </c>
+      <c r="B17" s="12">
+        <f>IF(ISNUMBER($B$16),$B$6*$B$14/$B$16,"–")</f>
+        <v/>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Hodnocení</t>
+        </is>
+      </c>
+      <c r="B18" s="14">
+        <f>IF(ISNUMBER($B$17),IF($B$17&lt;=$B$9,"OK","CHYBA – překročeno"),"–")</f>
+        <v/>
+      </c>
+      <c r="C18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Výkon při startu</t>
+        </is>
+      </c>
+      <c r="B19" s="10">
+        <f>$B$6*$B$5/1000</f>
+        <v/>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Ztráty v kabelu při startu</t>
+        </is>
+      </c>
+      <c r="B20" s="15">
+        <f>IF(ISNUMBER($B$16),$B$6^2*$B$14/$B$16,"–")</f>
+        <v/>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Zbývá napětí na startéru (bez poklesu baterie)</t>
+        </is>
+      </c>
+      <c r="B21" s="12">
+        <f>IF(ISNUMBER($B$17),$B$5-$B$17,"–")</f>
+        <v/>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B18">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>ISNUMBER(SEARCH("OK",B18))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>ISNUMBER(SEARCH("CHYBA",B18))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>ISNUMBER(SEARCH("POZOR",B18))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"12,24,48"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2665,7 +3344,7 @@
           <t>Energie baterie</t>
         </is>
       </c>
-      <c r="B11" s="20">
+      <c r="B11" s="23">
         <f>$B$5*$B$6</f>
         <v/>
       </c>
@@ -2681,7 +3360,7 @@
           <t>Využitelná energie</t>
         </is>
       </c>
-      <c r="B12" s="20">
+      <c r="B12" s="23">
         <f>$B$11*$B$7/100</f>
         <v/>
       </c>
@@ -2729,7 +3408,7 @@
           <t>Potřebná kapacita pro požadovanou výdrž</t>
         </is>
       </c>
-      <c r="B15" s="21">
+      <c r="B15" s="24">
         <f>$B$8*$B$10/($B$5*$B$7/100*$B$9/100)</f>
         <v/>
       </c>
@@ -3213,7 +3892,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3774,7 +4453,7 @@
           <t>Denní výnos (odhad, ztráty 25 %)</t>
         </is>
       </c>
-      <c r="B42" s="20">
+      <c r="B42" s="23">
         <f>$B$31*$B$34*0.75</f>
         <v/>
       </c>
@@ -3875,7 +4554,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3939,18 +4618,18 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>LED osvětlení</t>
         </is>
       </c>
-      <c r="B5" s="23" t="n">
+      <c r="B5" s="25" t="n">
         <v>24</v>
       </c>
-      <c r="C5" s="23" t="n">
+      <c r="C5" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="25" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="8">
@@ -3963,18 +4642,18 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>Kompresorová chladnička</t>
         </is>
       </c>
-      <c r="B6" s="23" t="n">
+      <c r="B6" s="25" t="n">
         <v>45</v>
       </c>
-      <c r="C6" s="23" t="n">
+      <c r="C6" s="25" t="n">
         <v>8</v>
       </c>
-      <c r="D6" s="23" t="n">
+      <c r="D6" s="25" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="8">
@@ -3987,18 +4666,18 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>Vodní čerpadlo</t>
         </is>
       </c>
-      <c r="B7" s="23" t="n">
+      <c r="B7" s="25" t="n">
         <v>60</v>
       </c>
-      <c r="C7" s="23" t="n">
+      <c r="C7" s="25" t="n">
         <v>0.3</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="25" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="8">
@@ -4011,18 +4690,18 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="25" t="inlineStr">
         <is>
           <t>Notebook + telefony</t>
         </is>
       </c>
-      <c r="B8" s="23" t="n">
+      <c r="B8" s="25" t="n">
         <v>60</v>
       </c>
-      <c r="C8" s="23" t="n">
+      <c r="C8" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="23" t="n">
+      <c r="D8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="8">
@@ -4035,18 +4714,18 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>Ventilátor</t>
         </is>
       </c>
-      <c r="B9" s="23" t="n">
+      <c r="B9" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="C9" s="23" t="n">
+      <c r="C9" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="8">
@@ -4059,10 +4738,10 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="inlineStr"/>
-      <c r="B10" s="23" t="n"/>
-      <c r="C10" s="23" t="n"/>
-      <c r="D10" s="23" t="n"/>
+      <c r="A10" s="25" t="inlineStr"/>
+      <c r="B10" s="25" t="n"/>
+      <c r="C10" s="25" t="n"/>
+      <c r="D10" s="25" t="n"/>
       <c r="E10" s="8">
         <f>IF(B10="","",B10*C10*D10)</f>
         <v/>
@@ -4073,10 +4752,10 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr"/>
-      <c r="B11" s="23" t="n"/>
-      <c r="C11" s="23" t="n"/>
-      <c r="D11" s="23" t="n"/>
+      <c r="A11" s="25" t="inlineStr"/>
+      <c r="B11" s="25" t="n"/>
+      <c r="C11" s="25" t="n"/>
+      <c r="D11" s="25" t="n"/>
       <c r="E11" s="8">
         <f>IF(B11="","",B11*C11*D11)</f>
         <v/>
@@ -4087,10 +4766,10 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr"/>
-      <c r="B12" s="23" t="n"/>
-      <c r="C12" s="23" t="n"/>
-      <c r="D12" s="23" t="n"/>
+      <c r="A12" s="25" t="inlineStr"/>
+      <c r="B12" s="25" t="n"/>
+      <c r="C12" s="25" t="n"/>
+      <c r="D12" s="25" t="n"/>
       <c r="E12" s="8">
         <f>IF(B12="","",B12*C12*D12)</f>
         <v/>
@@ -4101,10 +4780,10 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr"/>
-      <c r="B13" s="23" t="n"/>
-      <c r="C13" s="23" t="n"/>
-      <c r="D13" s="23" t="n"/>
+      <c r="A13" s="25" t="inlineStr"/>
+      <c r="B13" s="25" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
       <c r="E13" s="8">
         <f>IF(B13="","",B13*C13*D13)</f>
         <v/>
@@ -4115,10 +4794,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="inlineStr"/>
-      <c r="B14" s="23" t="n"/>
-      <c r="C14" s="23" t="n"/>
-      <c r="D14" s="23" t="n"/>
+      <c r="A14" s="25" t="inlineStr"/>
+      <c r="B14" s="25" t="n"/>
+      <c r="C14" s="25" t="n"/>
+      <c r="D14" s="25" t="n"/>
       <c r="E14" s="8">
         <f>IF(B14="","",B14*C14*D14)</f>
         <v/>
@@ -4129,10 +4808,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr"/>
-      <c r="B15" s="23" t="n"/>
-      <c r="C15" s="23" t="n"/>
-      <c r="D15" s="23" t="n"/>
+      <c r="A15" s="25" t="inlineStr"/>
+      <c r="B15" s="25" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
       <c r="E15" s="8">
         <f>IF(B15="","",B15*C15*D15)</f>
         <v/>
@@ -4143,10 +4822,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="inlineStr"/>
-      <c r="B16" s="23" t="n"/>
-      <c r="C16" s="23" t="n"/>
-      <c r="D16" s="23" t="n"/>
+      <c r="A16" s="25" t="inlineStr"/>
+      <c r="B16" s="25" t="n"/>
+      <c r="C16" s="25" t="n"/>
+      <c r="D16" s="25" t="n"/>
       <c r="E16" s="8">
         <f>IF(B16="","",B16*C16*D16)</f>
         <v/>
@@ -4233,7 +4912,7 @@
           <t>Spotřeba za den</t>
         </is>
       </c>
-      <c r="B23" s="20">
+      <c r="B23" s="23">
         <f>SUM(E5:E16)</f>
         <v/>
       </c>
@@ -4297,7 +4976,7 @@
           <t>Kapacita baterie pro zadané dny</t>
         </is>
       </c>
-      <c r="B27" s="21">
+      <c r="B27" s="24">
         <f>$B$23*$B$19/($B$18*$B$20/100*$B$21/100)</f>
         <v/>
       </c>
@@ -4329,7 +5008,7 @@
           <t>Solár pro pokrytí denní spotřeby</t>
         </is>
       </c>
-      <c r="B29" s="21">
+      <c r="B29" s="24">
         <f>$B$23/($B$22*0.75*$B$21/100)</f>
         <v/>
       </c>
@@ -4520,7 +5199,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4546,7 +5225,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>Typická napětí podle soustavy (násobek pro 12/24/48 V)</t>
         </is>
@@ -4869,7 +5548,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Průřez → trvalý proud → max. pojistka</t>
         </is>
@@ -4891,7 +5570,7 @@
           <t>max pojistka A</t>
         </is>
       </c>
-      <c r="F17" s="24" t="inlineStr">
+      <c r="F17" s="20" t="inlineStr">
         <is>
           <t>Značení svorek (DIN 72552)</t>
         </is>
@@ -5204,7 +5883,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="24" t="inlineStr">
+      <c r="A34" s="20" t="inlineStr">
         <is>
           <t>AWG → mm²</t>
         </is>
@@ -5231,11 +5910,11 @@
       <c r="A36" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="B36" s="25">
+      <c r="B36" s="26">
         <f>0.127*92^((36-24)/39)</f>
         <v/>
       </c>
-      <c r="C36" s="25">
+      <c r="C36" s="26">
         <f>PI()/4*B36^2</f>
         <v/>
       </c>
@@ -5244,11 +5923,11 @@
       <c r="A37" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="B37" s="25">
+      <c r="B37" s="26">
         <f>0.127*92^((36-22)/39)</f>
         <v/>
       </c>
-      <c r="C37" s="25">
+      <c r="C37" s="26">
         <f>PI()/4*B37^2</f>
         <v/>
       </c>
@@ -5257,11 +5936,11 @@
       <c r="A38" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="B38" s="25">
+      <c r="B38" s="26">
         <f>0.127*92^((36-20)/39)</f>
         <v/>
       </c>
-      <c r="C38" s="25">
+      <c r="C38" s="26">
         <f>PI()/4*B38^2</f>
         <v/>
       </c>
@@ -5270,11 +5949,11 @@
       <c r="A39" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="B39" s="25">
+      <c r="B39" s="26">
         <f>0.127*92^((36-18)/39)</f>
         <v/>
       </c>
-      <c r="C39" s="25">
+      <c r="C39" s="26">
         <f>PI()/4*B39^2</f>
         <v/>
       </c>
@@ -5283,11 +5962,11 @@
       <c r="A40" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="B40" s="25">
+      <c r="B40" s="26">
         <f>0.127*92^((36-16)/39)</f>
         <v/>
       </c>
-      <c r="C40" s="25">
+      <c r="C40" s="26">
         <f>PI()/4*B40^2</f>
         <v/>
       </c>
@@ -5296,11 +5975,11 @@
       <c r="A41" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B41" s="25">
+      <c r="B41" s="26">
         <f>0.127*92^((36-14)/39)</f>
         <v/>
       </c>
-      <c r="C41" s="25">
+      <c r="C41" s="26">
         <f>PI()/4*B41^2</f>
         <v/>
       </c>
@@ -5309,11 +5988,11 @@
       <c r="A42" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B42" s="25">
+      <c r="B42" s="26">
         <f>0.127*92^((36-12)/39)</f>
         <v/>
       </c>
-      <c r="C42" s="25">
+      <c r="C42" s="26">
         <f>PI()/4*B42^2</f>
         <v/>
       </c>
@@ -5322,11 +6001,11 @@
       <c r="A43" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B43" s="25">
+      <c r="B43" s="26">
         <f>0.127*92^((36-10)/39)</f>
         <v/>
       </c>
-      <c r="C43" s="25">
+      <c r="C43" s="26">
         <f>PI()/4*B43^2</f>
         <v/>
       </c>
@@ -5335,11 +6014,11 @@
       <c r="A44" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B44" s="25">
+      <c r="B44" s="26">
         <f>0.127*92^((36-8)/39)</f>
         <v/>
       </c>
-      <c r="C44" s="25">
+      <c r="C44" s="26">
         <f>PI()/4*B44^2</f>
         <v/>
       </c>
@@ -5348,11 +6027,11 @@
       <c r="A45" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B45" s="25">
+      <c r="B45" s="26">
         <f>0.127*92^((36-6)/39)</f>
         <v/>
       </c>
-      <c r="C45" s="25">
+      <c r="C45" s="26">
         <f>PI()/4*B45^2</f>
         <v/>
       </c>
@@ -5361,11 +6040,11 @@
       <c r="A46" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B46" s="25">
+      <c r="B46" s="26">
         <f>0.127*92^((36-4)/39)</f>
         <v/>
       </c>
-      <c r="C46" s="25">
+      <c r="C46" s="26">
         <f>PI()/4*B46^2</f>
         <v/>
       </c>
@@ -5374,11 +6053,11 @@
       <c r="A47" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B47" s="25">
+      <c r="B47" s="26">
         <f>0.127*92^((36-2)/39)</f>
         <v/>
       </c>
-      <c r="C47" s="25">
+      <c r="C47" s="26">
         <f>PI()/4*B47^2</f>
         <v/>
       </c>
@@ -5387,11 +6066,11 @@
       <c r="A48" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B48" s="25">
+      <c r="B48" s="26">
         <f>0.127*92^((36-1)/39)</f>
         <v/>
       </c>
-      <c r="C48" s="25">
+      <c r="C48" s="26">
         <f>PI()/4*B48^2</f>
         <v/>
       </c>
@@ -5402,11 +6081,11 @@
           <t>1/0</t>
         </is>
       </c>
-      <c r="B49" s="25">
+      <c r="B49" s="26">
         <f>0.127*92^((36-0)/39)</f>
         <v/>
       </c>
-      <c r="C49" s="25">
+      <c r="C49" s="26">
         <f>PI()/4*B49^2</f>
         <v/>
       </c>
@@ -5417,11 +6096,11 @@
           <t>2/0</t>
         </is>
       </c>
-      <c r="B50" s="25">
+      <c r="B50" s="26">
         <f>0.127*92^((36--1)/39)</f>
         <v/>
       </c>
-      <c r="C50" s="25">
+      <c r="C50" s="26">
         <f>PI()/4*B50^2</f>
         <v/>
       </c>
@@ -5432,11 +6111,11 @@
           <t>3/0</t>
         </is>
       </c>
-      <c r="B51" s="25">
+      <c r="B51" s="26">
         <f>0.127*92^((36--2)/39)</f>
         <v/>
       </c>
-      <c r="C51" s="25">
+      <c r="C51" s="26">
         <f>PI()/4*B51^2</f>
         <v/>
       </c>
@@ -5447,11 +6126,11 @@
           <t>4/0</t>
         </is>
       </c>
-      <c r="B52" s="25">
+      <c r="B52" s="26">
         <f>0.127*92^((36--3)/39)</f>
         <v/>
       </c>
-      <c r="C52" s="25">
+      <c r="C52" s="26">
         <f>PI()/4*B52^2</f>
         <v/>
       </c>
@@ -5459,160 +6138,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Check nový okruh</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Instalace nového spotřebiče / okruhu</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="24" t="inlineStr">
-        <is>
-          <t>Bod</t>
-        </is>
-      </c>
-      <c r="B4" s="24" t="inlineStr">
-        <is>
-          <t>Splněno (x)</t>
-        </is>
-      </c>
-      <c r="C4" s="24" t="inlineStr">
-        <is>
-          <t>Poznámka</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>Určen trvalý a špičkový proud spotřebiče</t>
-        </is>
-      </c>
-      <c r="B5" s="27" t="n"/>
-      <c r="C5" s="8" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="26" t="inlineStr">
-        <is>
-          <t>Pojistka nebo jistič co nejblíž ke zdroji (baterii), dimenzovaná na kabel</t>
-        </is>
-      </c>
-      <c r="B6" s="27" t="n"/>
-      <c r="C6" s="8" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="26" t="inlineStr">
-        <is>
-          <t>Průřez zkontrolován na úbytek napětí i na trvalý proud</t>
-        </is>
-      </c>
-      <c r="B7" s="27" t="n"/>
-      <c r="C7" s="8" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="26" t="inlineStr">
-        <is>
-          <t>Kabel odolný teplu a oděru, ochranný vlnovec, průchodky v plechu</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="n"/>
-      <c r="C8" s="8" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="26" t="inlineStr">
-        <is>
-          <t>Kvalitní lisované koncovky a spoje, správná velikost oka</t>
-        </is>
-      </c>
-      <c r="B9" s="27" t="n"/>
-      <c r="C9" s="8" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="26" t="inlineStr">
-        <is>
-          <t>Velké zátěže spínány přes relé / stykač</t>
-        </is>
-      </c>
-      <c r="B10" s="27" t="n"/>
-      <c r="C10" s="8" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="26" t="inlineStr">
-        <is>
-          <t>Kostrový spoj čistý, kov na kov, zajištěn proti uvolnění</t>
-        </is>
-      </c>
-      <c r="B11" s="27" t="n"/>
-      <c r="C11" s="8" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t>Spoje utaženy předepsaným momentem, svorky zakryty proti zkratu</t>
-        </is>
-      </c>
-      <c r="B12" s="27" t="n"/>
-      <c r="C12" s="8" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="26" t="inlineStr">
-        <is>
-          <t>Změřen úbytek napětí na plus i mínus pod zátěží</t>
-        </is>
-      </c>
-      <c r="B13" s="27" t="n"/>
-      <c r="C13" s="8" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="26" t="inlineStr">
-        <is>
-          <t>Zákres do schématu, kabely označeny</t>
-        </is>
-      </c>
-      <c r="B14" s="27" t="n"/>
-      <c r="C14" s="8" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="24">
-        <f>"Splněno "&amp;COUNTIF(B5:B14,"x")&amp;" z 10"</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="A5:B14">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$B5="x"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation sqref="B5 B6 B7 B8 B9 B10 B11 B12 B13 B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"x,"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>